<commit_message>
Long awaited update (pre cleaning)
</commit_message>
<xml_diff>
--- a/MATLAB/R14_Session_Metadata.xlsx
+++ b/MATLAB/R14_Session_Metadata.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/266ba68961b083a3/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Research\Encoder_Modeling\Encoder_Analysis\MATLAB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="555" documentId="8_{D768D4DC-9050-4594-B0B4-27F73FF04D73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF2120A0-FF87-4424-A16C-BB20C82FC2D1}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9A0F111-43D3-4617-8F59-D25F7FA50B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="0" windowWidth="29040" windowHeight="15720" xr2:uid="{9F7DED80-7A5A-4B53-A7F0-4EB3D3DD409C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$F$1:$F$52</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="66">
   <si>
     <t>Animal</t>
   </si>
@@ -231,6 +234,9 @@
   </si>
   <si>
     <t>To_include</t>
+  </si>
+  <si>
+    <t>M1ALM</t>
   </si>
 </sst>
 </file>
@@ -276,7 +282,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -334,6 +340,12 @@
         <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -350,7 +362,7 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -366,6 +378,11 @@
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="2"/>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="11" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="2" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="3" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
@@ -384,10 +401,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -707,6 +720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29F00D00-CC66-47DC-B071-BC70103919D6}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -758,7 +772,7 @@
         <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="E2" t="s">
         <v>36</v>
@@ -787,7 +801,7 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="E3" t="s">
         <v>36</v>
@@ -816,7 +830,7 @@
         <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="E4" t="s">
         <v>36</v>
@@ -845,7 +859,7 @@
         <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="E5" t="s">
         <v>38</v>
@@ -863,7 +877,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>25</v>
       </c>
@@ -892,7 +906,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>25</v>
       </c>
@@ -932,7 +946,7 @@
         <v>10</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -948,35 +962,32 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>4</v>
+      <c r="A9" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
         <v>10</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" t="s">
-        <v>37</v>
+        <v>65</v>
       </c>
       <c r="F9">
         <v>1</v>
       </c>
       <c r="G9" s="8">
-        <v>0.41292142000425203</v>
+        <v>0.50114459111746901</v>
       </c>
       <c r="H9" s="8">
-        <v>0.42380452320960998</v>
-      </c>
-      <c r="I9" s="12" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+        <v>0.31110152170613697</v>
+      </c>
+      <c r="I9" s="13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
@@ -1005,7 +1016,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>4</v>
       </c>
@@ -1035,139 +1046,136 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>4</v>
+      <c r="A12" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="B12" t="s">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
-      </c>
-      <c r="E12" t="s">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="F12">
         <v>1</v>
       </c>
       <c r="G12" s="8">
-        <v>0.50043956147813096</v>
+        <v>0.52342228565002102</v>
       </c>
       <c r="H12" s="8">
-        <v>0.45014375729036898</v>
+        <v>0.36130216430634599</v>
       </c>
       <c r="I12" s="12" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>13</v>
+      <c r="A13" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
         <v>9</v>
       </c>
       <c r="D13" t="s">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="F13">
         <v>1</v>
       </c>
       <c r="G13" s="8">
+        <v>0.30100247763070198</v>
+      </c>
+      <c r="H13" s="8">
+        <v>0.57766878915386699</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14" s="8">
+        <v>0.51032059753129799</v>
+      </c>
+      <c r="H14" s="8">
+        <v>0.39920345678681501</v>
+      </c>
+      <c r="I14" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" t="s">
+        <v>65</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15" s="8">
         <v>0.40175846656233699</v>
       </c>
-      <c r="H13" s="8">
+      <c r="H15" s="8">
         <v>0.51025769539164001</v>
       </c>
-      <c r="I13" s="13" t="s">
+      <c r="I15" s="13" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" t="s">
-        <v>35</v>
-      </c>
-      <c r="F14">
-        <v>1</v>
-      </c>
-      <c r="G14" s="8">
-        <v>0.49183320147695297</v>
-      </c>
-      <c r="H14" s="8">
-        <v>0.44322202952151302</v>
-      </c>
-      <c r="I14" s="12" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" t="s">
-        <v>9</v>
-      </c>
-      <c r="D15" t="s">
-        <v>35</v>
-      </c>
-      <c r="F15">
-        <v>1</v>
-      </c>
-      <c r="G15" s="8">
-        <v>0.648602590171516</v>
-      </c>
-      <c r="H15" s="8">
-        <v>0.50680373219873998</v>
-      </c>
-      <c r="I15" s="12" t="s">
-        <v>46</v>
-      </c>
-    </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>13</v>
+      <c r="A16" s="7" t="s">
+        <v>31</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="C16" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D16" t="s">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="F16">
         <v>1</v>
       </c>
       <c r="G16" s="8">
-        <v>0.54828216793503703</v>
+        <v>0.40559089530613601</v>
       </c>
       <c r="H16" s="8">
-        <v>0.30049412545439502</v>
-      </c>
-      <c r="I16" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+        <v>0.45241814570834799</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>25</v>
       </c>
@@ -1196,7 +1204,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>25</v>
       </c>
@@ -1226,64 +1234,64 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B19" t="s">
-        <v>21</v>
-      </c>
-      <c r="C19" t="s">
-        <v>9</v>
+      <c r="A19" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>10</v>
       </c>
       <c r="D19" t="s">
-        <v>35</v>
-      </c>
-      <c r="E19" t="s">
-        <v>36</v>
-      </c>
-      <c r="F19">
-        <v>1</v>
-      </c>
-      <c r="G19" s="8">
-        <v>0.45466970184186201</v>
-      </c>
-      <c r="H19" s="8">
-        <v>0.34638139832360398</v>
-      </c>
-      <c r="I19" t="s">
-        <v>48</v>
+        <v>65</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="F19" s="15">
+        <v>1</v>
+      </c>
+      <c r="G19" s="16">
+        <v>0.41292142000425203</v>
+      </c>
+      <c r="H19" s="16">
+        <v>0.42380452320960998</v>
+      </c>
+      <c r="I19" s="17" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B20" t="s">
-        <v>22</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="A20" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="C20" s="15" t="s">
         <v>10</v>
       </c>
       <c r="D20" t="s">
-        <v>35</v>
-      </c>
-      <c r="E20" t="s">
-        <v>38</v>
-      </c>
-      <c r="F20">
-        <v>1</v>
-      </c>
-      <c r="G20" s="8">
-        <v>0.367997223460861</v>
-      </c>
-      <c r="H20" s="8">
-        <v>0.34881455596535199</v>
-      </c>
-      <c r="I20" s="13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="F20" s="15">
+        <v>1</v>
+      </c>
+      <c r="G20" s="16">
+        <v>0.50043956147813096</v>
+      </c>
+      <c r="H20" s="16">
+        <v>0.45014375729036898</v>
+      </c>
+      <c r="I20" s="17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>25</v>
       </c>
@@ -1312,7 +1320,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>25</v>
       </c>
@@ -1342,93 +1350,87 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" t="s">
-        <v>26</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="A23" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" s="15" t="s">
         <v>9</v>
       </c>
       <c r="D23" t="s">
-        <v>35</v>
-      </c>
-      <c r="E23" t="s">
-        <v>36</v>
-      </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-      <c r="G23" s="8">
-        <v>0.41908114302477001</v>
-      </c>
-      <c r="H23" s="8">
-        <v>0.37550276527717702</v>
-      </c>
-      <c r="I23" s="14" t="s">
-        <v>52</v>
+        <v>65</v>
+      </c>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15">
+        <v>1</v>
+      </c>
+      <c r="G23" s="16">
+        <v>0.40175846656233699</v>
+      </c>
+      <c r="H23" s="16">
+        <v>0.51025769539164001</v>
+      </c>
+      <c r="I23" s="18" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24" t="s">
-        <v>27</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="A24" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="C24" s="15" t="s">
         <v>9</v>
       </c>
       <c r="D24" t="s">
-        <v>35</v>
-      </c>
-      <c r="E24" t="s">
-        <v>36</v>
-      </c>
-      <c r="F24">
-        <v>1</v>
-      </c>
-      <c r="G24" s="8">
-        <v>0.533556288668249</v>
-      </c>
-      <c r="H24" s="8">
-        <v>0.382416788847592</v>
-      </c>
-      <c r="I24" s="14" t="s">
-        <v>52</v>
+        <v>65</v>
+      </c>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15">
+        <v>1</v>
+      </c>
+      <c r="G24" s="16">
+        <v>0.49183320147695297</v>
+      </c>
+      <c r="H24" s="16">
+        <v>0.44322202952151302</v>
+      </c>
+      <c r="I24" s="17" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25" t="s">
-        <v>28</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="A25" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="15" t="s">
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>35</v>
-      </c>
-      <c r="E25" t="s">
-        <v>38</v>
-      </c>
-      <c r="F25">
-        <v>1</v>
-      </c>
-      <c r="G25" s="8">
-        <v>0.44163248149254702</v>
-      </c>
-      <c r="H25" s="8">
-        <v>0.45883374112124098</v>
-      </c>
-      <c r="I25" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15">
+        <v>1</v>
+      </c>
+      <c r="G25" s="16">
+        <v>0.648602590171516</v>
+      </c>
+      <c r="H25" s="16">
+        <v>0.50680373219873998</v>
+      </c>
+      <c r="I25" s="17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>24</v>
       </c>
@@ -1458,110 +1460,120 @@
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A27" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B27" t="s">
-        <v>32</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="A27" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="15" t="s">
         <v>9</v>
       </c>
       <c r="D27" t="s">
-        <v>35</v>
-      </c>
-      <c r="F27">
-        <v>1</v>
-      </c>
-      <c r="G27" s="8">
-        <v>0.45867290466997201</v>
-      </c>
-      <c r="H27" s="8">
-        <v>0.50883334464178698</v>
-      </c>
-      <c r="I27" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15">
+        <v>1</v>
+      </c>
+      <c r="G27" s="16">
+        <v>0.54828216793503703</v>
+      </c>
+      <c r="H27" s="16">
+        <v>0.30049412545439502</v>
+      </c>
+      <c r="I27" s="17" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A28" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" t="s">
+        <v>65</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F28" s="15">
+        <v>1</v>
+      </c>
+      <c r="G28" s="16">
+        <v>0.45466970184186201</v>
+      </c>
+      <c r="H28" s="16">
+        <v>0.34638139832360398</v>
+      </c>
+      <c r="I28" s="15" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" t="s">
+        <v>65</v>
+      </c>
+      <c r="E29" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F29" s="15">
+        <v>1</v>
+      </c>
+      <c r="G29" s="16">
+        <v>0.367997223460861</v>
+      </c>
+      <c r="H29" s="16">
+        <v>0.34881455596535199</v>
+      </c>
+      <c r="I29" s="18" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A28" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28" t="s">
-        <v>32</v>
-      </c>
-      <c r="C28" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" t="s">
-        <v>35</v>
-      </c>
-      <c r="F28">
-        <v>1</v>
-      </c>
-      <c r="G28" s="8">
-        <v>0.32217939946207802</v>
-      </c>
-      <c r="H28" s="8">
-        <v>0.34194752353984298</v>
-      </c>
-      <c r="I28" s="14" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A29" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" t="s">
-        <v>33</v>
-      </c>
-      <c r="C29" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" t="s">
-        <v>35</v>
-      </c>
-      <c r="F29">
-        <v>1</v>
-      </c>
-      <c r="G29" s="8">
-        <v>0.51763345083014101</v>
-      </c>
-      <c r="H29" s="8">
-        <v>0.334503175977513</v>
-      </c>
-      <c r="I29" s="12" t="s">
-        <v>46</v>
-      </c>
-    </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" t="s">
-        <v>42</v>
-      </c>
-      <c r="C30" t="s">
-        <v>10</v>
+      <c r="A30" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>9</v>
       </c>
       <c r="D30" t="s">
-        <v>35</v>
-      </c>
-      <c r="F30">
-        <v>1</v>
-      </c>
-      <c r="G30" s="8">
-        <v>0.30721605108922001</v>
-      </c>
-      <c r="H30" s="8">
-        <v>0.48047872813921599</v>
-      </c>
-      <c r="I30" s="12" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F30" s="15">
+        <v>1</v>
+      </c>
+      <c r="G30" s="16">
+        <v>0.41908114302477001</v>
+      </c>
+      <c r="H30" s="16">
+        <v>0.37550276527717702</v>
+      </c>
+      <c r="I30" s="19" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
         <v>30</v>
       </c>
@@ -1587,7 +1599,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>31</v>
       </c>
@@ -1613,7 +1625,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
         <v>31</v>
       </c>
@@ -1639,7 +1651,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
         <v>31</v>
       </c>
@@ -1665,7 +1677,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
         <v>31</v>
       </c>
@@ -1691,7 +1703,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="7" t="s">
         <v>31</v>
       </c>
@@ -1718,84 +1730,91 @@
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D37" t="s">
+        <v>65</v>
+      </c>
+      <c r="E37" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F37" s="15">
+        <v>1</v>
+      </c>
+      <c r="G37" s="16">
+        <v>0.533556288668249</v>
+      </c>
+      <c r="H37" s="16">
+        <v>0.382416788847592</v>
+      </c>
+      <c r="I37" s="19" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38" t="s">
+        <v>65</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F38" s="15">
+        <v>1</v>
+      </c>
+      <c r="G38" s="16">
+        <v>0.44163248149254702</v>
+      </c>
+      <c r="H38" s="16">
+        <v>0.45883374112124098</v>
+      </c>
+      <c r="I38" s="17" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B37" t="s">
-        <v>33</v>
-      </c>
-      <c r="C37" t="s">
-        <v>10</v>
-      </c>
-      <c r="D37" t="s">
-        <v>34</v>
-      </c>
-      <c r="F37">
-        <v>1</v>
-      </c>
-      <c r="G37" s="8">
-        <v>0.50114459111746901</v>
-      </c>
-      <c r="H37" s="8">
-        <v>0.31110152170613697</v>
-      </c>
-      <c r="I37" s="13" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A38" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B38" t="s">
-        <v>42</v>
-      </c>
-      <c r="C38" t="s">
-        <v>9</v>
-      </c>
-      <c r="D38" t="s">
-        <v>34</v>
-      </c>
-      <c r="F38">
-        <v>1</v>
-      </c>
-      <c r="G38" s="8">
-        <v>0.52342228565002102</v>
-      </c>
-      <c r="H38" s="8">
-        <v>0.36130216430634599</v>
-      </c>
-      <c r="I38" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A39" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="B39" t="s">
-        <v>43</v>
-      </c>
-      <c r="C39" t="s">
+      <c r="B39" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C39" s="15" t="s">
         <v>9</v>
       </c>
       <c r="D39" t="s">
-        <v>34</v>
-      </c>
-      <c r="F39">
-        <v>1</v>
-      </c>
-      <c r="G39" s="8">
-        <v>0.30100247763070198</v>
-      </c>
-      <c r="H39" s="8">
-        <v>0.57766878915386699</v>
-      </c>
-      <c r="I39" s="14" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15">
+        <v>1</v>
+      </c>
+      <c r="G39" s="16">
+        <v>0.45867290466997201</v>
+      </c>
+      <c r="H39" s="16">
+        <v>0.50883334464178698</v>
+      </c>
+      <c r="I39" s="18" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
         <v>31</v>
       </c>
@@ -1822,84 +1841,87 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A41" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B41" t="s">
+      <c r="A41" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D41" t="s">
+        <v>65</v>
+      </c>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15">
+        <v>1</v>
+      </c>
+      <c r="G41" s="16">
+        <v>0.32217939946207802</v>
+      </c>
+      <c r="H41" s="16">
+        <v>0.34194752353984298</v>
+      </c>
+      <c r="I41" s="19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B42" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="C41" t="s">
-        <v>9</v>
-      </c>
-      <c r="D41" t="s">
-        <v>34</v>
-      </c>
-      <c r="F41">
-        <v>1</v>
-      </c>
-      <c r="G41" s="8">
-        <v>0.51032059753129799</v>
-      </c>
-      <c r="H41" s="8">
-        <v>0.39920345678681501</v>
-      </c>
-      <c r="I41" s="13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A42" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B42" t="s">
+      <c r="C42" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42" t="s">
+        <v>65</v>
+      </c>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15">
+        <v>1</v>
+      </c>
+      <c r="G42" s="16">
+        <v>0.51763345083014101</v>
+      </c>
+      <c r="H42" s="16">
+        <v>0.334503175977513</v>
+      </c>
+      <c r="I42" s="17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B43" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C42" t="s">
-        <v>9</v>
-      </c>
-      <c r="D42" t="s">
-        <v>34</v>
-      </c>
-      <c r="F42">
-        <v>1</v>
-      </c>
-      <c r="G42" s="8">
-        <v>0.40175846656233699</v>
-      </c>
-      <c r="H42" s="8">
-        <v>0.51025769539164001</v>
-      </c>
-      <c r="I42" s="13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A43" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B43" t="s">
-        <v>43</v>
-      </c>
-      <c r="C43" t="s">
+      <c r="C43" s="15" t="s">
         <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>34</v>
-      </c>
-      <c r="F43">
-        <v>1</v>
-      </c>
-      <c r="G43" s="8">
-        <v>0.40559089530613601</v>
-      </c>
-      <c r="H43" s="8">
-        <v>0.45241814570834799</v>
-      </c>
-      <c r="I43" s="14" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+      <c r="E43" s="15"/>
+      <c r="F43" s="15">
+        <v>1</v>
+      </c>
+      <c r="G43" s="16">
+        <v>0.30721605108922001</v>
+      </c>
+      <c r="H43" s="16">
+        <v>0.48047872813921599</v>
+      </c>
+      <c r="I43" s="17" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
         <v>31</v>
       </c>
@@ -1925,7 +1947,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>25</v>
       </c>
@@ -1954,7 +1976,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>25</v>
       </c>
@@ -2070,7 +2092,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
         <v>24</v>
       </c>
@@ -2099,7 +2121,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
         <v>24</v>
       </c>
@@ -2128,7 +2150,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
         <v>24</v>
       </c>
@@ -2158,7 +2180,14 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I52">
+  <autoFilter ref="F1:F52" xr:uid="{29F00D00-CC66-47DC-B071-BC70103919D6}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I49">
     <sortCondition ref="D1:D52"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>